<commit_message>
Race 2 points, race 3 selection
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="12" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="15" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -279,7 +279,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -291,6 +291,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5757,6 +5763,9 @@
       <c r="D1" s="3">
         <v>2</v>
       </c>
+      <c r="E1" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5769,6 +5778,9 @@
         <v>21</v>
       </c>
       <c r="D2" s="2">
+        <v>-10</v>
+      </c>
+      <c r="E2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5783,6 +5795,9 @@
         <v>-14</v>
       </c>
       <c r="D3" s="2">
+        <v>-7</v>
+      </c>
+      <c r="E3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5797,6 +5812,9 @@
         <v>39</v>
       </c>
       <c r="D4" s="2">
+        <v>45</v>
+      </c>
+      <c r="E4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5811,6 +5829,9 @@
         <v>32</v>
       </c>
       <c r="D5" s="2">
+        <v>68</v>
+      </c>
+      <c r="E5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5825,6 +5846,9 @@
         <v>50</v>
       </c>
       <c r="D6" s="2">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5839,6 +5863,9 @@
         <v>-8</v>
       </c>
       <c r="D7" s="2">
+        <v>19</v>
+      </c>
+      <c r="E7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5853,6 +5880,9 @@
         <v>25</v>
       </c>
       <c r="D8" s="2">
+        <v>48</v>
+      </c>
+      <c r="E8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5867,6 +5897,9 @@
         <v>29</v>
       </c>
       <c r="D9" s="2">
+        <v>51</v>
+      </c>
+      <c r="E9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5881,6 +5914,9 @@
         <v>8</v>
       </c>
       <c r="D10" s="2">
+        <v>-7</v>
+      </c>
+      <c r="E10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5895,6 +5931,9 @@
         <v>9</v>
       </c>
       <c r="D11" s="2">
+        <v>28</v>
+      </c>
+      <c r="E11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5909,6 +5948,9 @@
         <v>5</v>
       </c>
       <c r="D12" s="2">
+        <v>35</v>
+      </c>
+      <c r="E12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5923,6 +5965,9 @@
         <v>15</v>
       </c>
       <c r="D13" s="2">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5937,6 +5982,9 @@
         <v>-14</v>
       </c>
       <c r="D14" s="2">
+        <v>-7</v>
+      </c>
+      <c r="E14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5951,6 +5999,9 @@
         <v>-23</v>
       </c>
       <c r="D15" s="2">
+        <v>-14</v>
+      </c>
+      <c r="E15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5965,6 +6016,9 @@
         <v>9</v>
       </c>
       <c r="D16" s="2">
+        <v>24</v>
+      </c>
+      <c r="E16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5979,6 +6033,9 @@
         <v>20</v>
       </c>
       <c r="D17" s="2">
+        <v>34</v>
+      </c>
+      <c r="E17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5993,6 +6050,9 @@
         <v>-20</v>
       </c>
       <c r="D18" s="2">
+        <v>7</v>
+      </c>
+      <c r="E18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6007,6 +6067,9 @@
         <v>13</v>
       </c>
       <c r="D19" s="2">
+        <v>-14</v>
+      </c>
+      <c r="E19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6021,6 +6084,9 @@
         <v>11</v>
       </c>
       <c r="D20" s="2">
+        <v>20</v>
+      </c>
+      <c r="E20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6035,6 +6101,9 @@
         <v>6</v>
       </c>
       <c r="D21" s="2">
+        <v>18</v>
+      </c>
+      <c r="E21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6049,6 +6118,9 @@
         <v>-16</v>
       </c>
       <c r="D22" s="2">
+        <v>3</v>
+      </c>
+      <c r="E22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6063,6 +6135,9 @@
         <v>4</v>
       </c>
       <c r="D23" s="2">
+        <v>20</v>
+      </c>
+      <c r="E23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6093,6 +6168,9 @@
       <c r="C1" s="3">
         <v>2</v>
       </c>
+      <c r="D1" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6102,6 +6180,9 @@
         <v>19</v>
       </c>
       <c r="C2" s="2">
+        <v>-7</v>
+      </c>
+      <c r="D2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6113,6 +6194,9 @@
         <v>69</v>
       </c>
       <c r="C3" s="2">
+        <v>119</v>
+      </c>
+      <c r="D3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6124,6 +6208,9 @@
         <v>42</v>
       </c>
       <c r="C4" s="2">
+        <v>45</v>
+      </c>
+      <c r="D4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6135,6 +6222,9 @@
         <v>96</v>
       </c>
       <c r="C5" s="2">
+        <v>115</v>
+      </c>
+      <c r="D5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6146,6 +6236,9 @@
         <v>20</v>
       </c>
       <c r="C6" s="2">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6157,6 +6250,9 @@
         <v>34</v>
       </c>
       <c r="C7" s="2">
+        <v>65</v>
+      </c>
+      <c r="D7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6168,6 +6264,9 @@
         <v>35</v>
       </c>
       <c r="C8" s="2">
+        <v>50</v>
+      </c>
+      <c r="D8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6179,6 +6278,9 @@
         <v>0</v>
       </c>
       <c r="C9" s="2">
+        <v>-4</v>
+      </c>
+      <c r="D9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6190,6 +6292,9 @@
         <v>-38</v>
       </c>
       <c r="C10" s="2">
+        <v>-20</v>
+      </c>
+      <c r="D10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6201,6 +6306,9 @@
         <v>22</v>
       </c>
       <c r="C11" s="2">
+        <v>45</v>
+      </c>
+      <c r="D11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6212,6 +6320,9 @@
         <v>-13</v>
       </c>
       <c r="C12" s="2">
+        <v>22</v>
+      </c>
+      <c r="D12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6240,6 +6351,9 @@
       <c r="D1" s="3">
         <v>2</v>
       </c>
+      <c r="E1" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -6254,7 +6368,9 @@
       <c r="D2" s="1">
         <v>27.1</v>
       </c>
-      <c r="E2" s="2"/>
+      <c r="E2" s="6">
+        <v>26.8</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -6269,6 +6385,9 @@
       <c r="D3" s="1">
         <v>25.2</v>
       </c>
+      <c r="E3" s="7">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -6283,6 +6402,9 @@
       <c r="D4" s="1">
         <v>27.7</v>
       </c>
+      <c r="E4" s="7">
+        <v>28</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -6297,6 +6419,9 @@
       <c r="D5" s="1">
         <v>23.5</v>
       </c>
+      <c r="E5" s="7">
+        <v>23.8</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -6311,6 +6436,9 @@
       <c r="D6" s="1">
         <v>28</v>
       </c>
+      <c r="E6" s="7">
+        <v>28.1</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -6325,6 +6453,9 @@
       <c r="D7" s="1">
         <v>14.5</v>
       </c>
+      <c r="E7" s="7">
+        <v>13.9</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -6339,7 +6470,9 @@
       <c r="D8" s="1">
         <v>22.6</v>
       </c>
-      <c r="E8" s="2"/>
+      <c r="E8" s="6">
+        <v>22.9</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -6354,6 +6487,9 @@
       <c r="D9" s="1">
         <v>23.1</v>
       </c>
+      <c r="E9" s="7">
+        <v>23.4</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -6368,7 +6504,9 @@
       <c r="D10" s="1">
         <v>11.4</v>
       </c>
-      <c r="E10" s="2"/>
+      <c r="E10" s="6">
+        <v>10.8</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -6383,6 +6521,9 @@
       <c r="D11" s="1">
         <v>11.6</v>
       </c>
+      <c r="E11" s="7">
+        <v>12.2</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -6397,7 +6538,9 @@
       <c r="D12" s="1">
         <v>6.3</v>
       </c>
-      <c r="E12" s="2"/>
+      <c r="E12" s="6">
+        <v>6.9</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -6412,6 +6555,9 @@
       <c r="D13" s="1">
         <v>6.8</v>
       </c>
+      <c r="E13" s="7">
+        <v>7.4</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -6426,6 +6572,9 @@
       <c r="D14" s="1">
         <v>9.4</v>
       </c>
+      <c r="E14" s="7">
+        <v>8.8</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -6440,6 +6589,9 @@
       <c r="D15" s="1">
         <v>7.4</v>
       </c>
+      <c r="E15" s="7">
+        <v>6.8</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -6454,6 +6606,9 @@
       <c r="D16" s="1">
         <v>7.9</v>
       </c>
+      <c r="E16" s="7">
+        <v>8.5</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -6468,6 +6623,9 @@
       <c r="D17" s="1">
         <v>8</v>
       </c>
+      <c r="E17" s="7">
+        <v>8.6</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -6482,6 +6640,9 @@
       <c r="D18" s="1">
         <v>6.2</v>
       </c>
+      <c r="E18" s="7">
+        <v>5.6</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -6496,6 +6657,9 @@
       <c r="D19" s="1">
         <v>7</v>
       </c>
+      <c r="E19" s="7">
+        <v>6.4</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -6510,7 +6674,9 @@
       <c r="D20" s="1">
         <v>12.2</v>
       </c>
-      <c r="E20" s="2"/>
+      <c r="E20" s="6">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -6525,6 +6691,9 @@
       <c r="D21" s="1">
         <v>6.4</v>
       </c>
+      <c r="E21" s="7">
+        <v>7</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -6539,6 +6708,9 @@
       <c r="D22" s="1">
         <v>5.3</v>
       </c>
+      <c r="E22" s="7">
+        <v>4.7</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -6552,6 +6724,9 @@
       </c>
       <c r="D23" s="1">
         <v>5.8</v>
+      </c>
+      <c r="E23" s="7">
+        <v>6.4</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -6581,6 +6756,9 @@
       <c r="C1" s="3">
         <v>2</v>
       </c>
+      <c r="D1" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6592,6 +6770,9 @@
       <c r="C2" s="1">
         <v>28.8</v>
       </c>
+      <c r="D2" s="7">
+        <v>28.5</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -6603,6 +6784,9 @@
       <c r="C3" s="1">
         <v>23.6</v>
       </c>
+      <c r="D3" s="7">
+        <v>23.9</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -6614,6 +6798,9 @@
       <c r="C4" s="1">
         <v>28.5</v>
       </c>
+      <c r="D4" s="7">
+        <v>28.8</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -6625,6 +6812,9 @@
       <c r="C5" s="1">
         <v>29.6</v>
       </c>
+      <c r="D5" s="7">
+        <v>29.9</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -6636,6 +6826,9 @@
       <c r="C6" s="1">
         <v>12.6</v>
       </c>
+      <c r="D6" s="7">
+        <v>13.2</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -6647,6 +6840,9 @@
       <c r="C7" s="1">
         <v>6.9</v>
       </c>
+      <c r="D7" s="7">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -6658,6 +6854,9 @@
       <c r="C8" s="1">
         <v>8</v>
       </c>
+      <c r="D8" s="7">
+        <v>8.6</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -6669,6 +6868,9 @@
       <c r="C9" s="1">
         <v>9.7</v>
       </c>
+      <c r="D9" s="7">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -6680,6 +6882,9 @@
       <c r="C10" s="1">
         <v>13.1</v>
       </c>
+      <c r="D10" s="7">
+        <v>13.7</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -6691,6 +6896,9 @@
       <c r="C11" s="1">
         <v>6</v>
       </c>
+      <c r="D11" s="7">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -6701,6 +6909,9 @@
       </c>
       <c r="C12" s="1">
         <v>5.4</v>
+      </c>
+      <c r="D12" s="7">
+        <v>5.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated points after race 3
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="15" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="13" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -5766,6 +5766,9 @@
       <c r="E1" s="3">
         <v>3</v>
       </c>
+      <c r="F1" s="3">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5781,6 +5784,9 @@
         <v>-10</v>
       </c>
       <c r="E2" s="2">
+        <v>24</v>
+      </c>
+      <c r="F2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5798,6 +5804,9 @@
         <v>-7</v>
       </c>
       <c r="E3" s="2">
+        <v>43</v>
+      </c>
+      <c r="F3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5815,6 +5824,9 @@
         <v>45</v>
       </c>
       <c r="E4" s="2">
+        <v>27</v>
+      </c>
+      <c r="F4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5832,6 +5844,9 @@
         <v>68</v>
       </c>
       <c r="E5" s="2">
+        <v>50</v>
+      </c>
+      <c r="F5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5849,6 +5864,9 @@
         <v>14</v>
       </c>
       <c r="E6" s="2">
+        <v>13</v>
+      </c>
+      <c r="F6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5866,6 +5884,9 @@
         <v>19</v>
       </c>
       <c r="E7" s="2">
+        <v>5</v>
+      </c>
+      <c r="F7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5883,6 +5904,9 @@
         <v>48</v>
       </c>
       <c r="E8" s="2">
+        <v>19</v>
+      </c>
+      <c r="F8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5900,6 +5924,9 @@
         <v>51</v>
       </c>
       <c r="E9" s="2">
+        <v>31</v>
+      </c>
+      <c r="F9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5917,6 +5944,9 @@
         <v>-7</v>
       </c>
       <c r="E10" s="2">
+        <v>-1</v>
+      </c>
+      <c r="F10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5934,6 +5964,9 @@
         <v>28</v>
       </c>
       <c r="E11" s="2">
+        <v>4</v>
+      </c>
+      <c r="F11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5951,6 +5984,9 @@
         <v>35</v>
       </c>
       <c r="E12" s="2">
+        <v>10</v>
+      </c>
+      <c r="F12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5968,6 +6004,9 @@
         <v>7</v>
       </c>
       <c r="E13" s="2">
+        <v>1</v>
+      </c>
+      <c r="F13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5985,6 +6024,9 @@
         <v>-7</v>
       </c>
       <c r="E14" s="2">
+        <v>4</v>
+      </c>
+      <c r="F14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6002,6 +6044,9 @@
         <v>-14</v>
       </c>
       <c r="E15" s="2">
+        <v>-17</v>
+      </c>
+      <c r="F15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6019,6 +6064,9 @@
         <v>24</v>
       </c>
       <c r="E16" s="2">
+        <v>9</v>
+      </c>
+      <c r="F16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6036,6 +6084,9 @@
         <v>34</v>
       </c>
       <c r="E17" s="2">
+        <v>-14</v>
+      </c>
+      <c r="F17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6053,6 +6104,9 @@
         <v>7</v>
       </c>
       <c r="E18" s="2">
+        <v>10</v>
+      </c>
+      <c r="F18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6070,6 +6124,9 @@
         <v>-14</v>
       </c>
       <c r="E19" s="2">
+        <v>3</v>
+      </c>
+      <c r="F19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6087,6 +6144,9 @@
         <v>20</v>
       </c>
       <c r="E20" s="2">
+        <v>14</v>
+      </c>
+      <c r="F20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6104,6 +6164,9 @@
         <v>18</v>
       </c>
       <c r="E21" s="2">
+        <v>4</v>
+      </c>
+      <c r="F21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6121,6 +6184,9 @@
         <v>3</v>
       </c>
       <c r="E22" s="2">
+        <v>2</v>
+      </c>
+      <c r="F22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6138,6 +6204,9 @@
         <v>20</v>
       </c>
       <c r="E23" s="2">
+        <v>4</v>
+      </c>
+      <c r="F23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6171,6 +6240,9 @@
       <c r="D1" s="3">
         <v>3</v>
       </c>
+      <c r="E1" s="3">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6183,6 +6255,9 @@
         <v>-7</v>
       </c>
       <c r="D2" s="2">
+        <v>72</v>
+      </c>
+      <c r="E2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6197,6 +6272,9 @@
         <v>119</v>
       </c>
       <c r="D3" s="2">
+        <v>75</v>
+      </c>
+      <c r="E3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6211,6 +6289,9 @@
         <v>45</v>
       </c>
       <c r="D4" s="2">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6225,6 +6306,9 @@
         <v>115</v>
       </c>
       <c r="D5" s="2">
+        <v>92</v>
+      </c>
+      <c r="E5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6239,6 +6323,9 @@
         <v>22</v>
       </c>
       <c r="D6" s="2">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6253,6 +6340,9 @@
         <v>65</v>
       </c>
       <c r="D7" s="2">
+        <v>-4</v>
+      </c>
+      <c r="E7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6267,6 +6357,9 @@
         <v>50</v>
       </c>
       <c r="D8" s="2">
+        <v>18</v>
+      </c>
+      <c r="E8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6281,6 +6374,9 @@
         <v>-4</v>
       </c>
       <c r="D9" s="2">
+        <v>23</v>
+      </c>
+      <c r="E9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6295,6 +6391,9 @@
         <v>-20</v>
       </c>
       <c r="D10" s="2">
+        <v>-12</v>
+      </c>
+      <c r="E10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6309,6 +6408,9 @@
         <v>45</v>
       </c>
       <c r="D11" s="2">
+        <v>25</v>
+      </c>
+      <c r="E11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6323,6 +6425,9 @@
         <v>22</v>
       </c>
       <c r="D12" s="2">
+        <v>5</v>
+      </c>
+      <c r="E12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6354,6 +6459,9 @@
       <c r="E1" s="3">
         <v>3</v>
       </c>
+      <c r="F1" s="3">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -6371,6 +6479,9 @@
       <c r="E2" s="6">
         <v>26.8</v>
       </c>
+      <c r="F2" s="6">
+        <v>26.5</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -6388,6 +6499,9 @@
       <c r="E3" s="7">
         <v>24.9</v>
       </c>
+      <c r="F3" s="7">
+        <v>24.6</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -6405,6 +6519,9 @@
       <c r="E4" s="7">
         <v>28</v>
       </c>
+      <c r="F4" s="7">
+        <v>28.3</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -6422,6 +6539,9 @@
       <c r="E5" s="7">
         <v>23.8</v>
       </c>
+      <c r="F5" s="7">
+        <v>24.1</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -6439,6 +6559,9 @@
       <c r="E6" s="7">
         <v>28.1</v>
       </c>
+      <c r="F6" s="7">
+        <v>28.1</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -6456,6 +6579,9 @@
       <c r="E7" s="7">
         <v>13.9</v>
       </c>
+      <c r="F7" s="7">
+        <v>13.3</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -6473,6 +6599,9 @@
       <c r="E8" s="6">
         <v>22.9</v>
       </c>
+      <c r="F8" s="6">
+        <v>23.2</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -6490,6 +6619,9 @@
       <c r="E9" s="7">
         <v>23.4</v>
       </c>
+      <c r="F9" s="7">
+        <v>23.7</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -6507,6 +6639,9 @@
       <c r="E10" s="6">
         <v>10.8</v>
       </c>
+      <c r="F10" s="6">
+        <v>10.2</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -6524,6 +6659,9 @@
       <c r="E11" s="7">
         <v>12.2</v>
       </c>
+      <c r="F11" s="7">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -6541,6 +6679,9 @@
       <c r="E12" s="6">
         <v>6.9</v>
       </c>
+      <c r="F12" s="6">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -6558,6 +6699,9 @@
       <c r="E13" s="7">
         <v>7.4</v>
       </c>
+      <c r="F13" s="7">
+        <v>7.6</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -6575,6 +6719,9 @@
       <c r="E14" s="7">
         <v>8.8</v>
       </c>
+      <c r="F14" s="7">
+        <v>8.2</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -6592,6 +6739,9 @@
       <c r="E15" s="7">
         <v>6.8</v>
       </c>
+      <c r="F15" s="7">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -6609,6 +6759,9 @@
       <c r="E16" s="7">
         <v>8.5</v>
       </c>
+      <c r="F16" s="7">
+        <v>9.1</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -6626,6 +6779,9 @@
       <c r="E17" s="7">
         <v>8.6</v>
       </c>
+      <c r="F17" s="7">
+        <v>9.2</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -6643,6 +6799,9 @@
       <c r="E18" s="7">
         <v>5.6</v>
       </c>
+      <c r="F18" s="7">
+        <v>5</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -6660,6 +6819,9 @@
       <c r="E19" s="7">
         <v>6.4</v>
       </c>
+      <c r="F19" s="7">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -6677,6 +6839,9 @@
       <c r="E20" s="6">
         <v>12.8</v>
       </c>
+      <c r="F20" s="6">
+        <v>13</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -6694,6 +6859,9 @@
       <c r="E21" s="7">
         <v>7</v>
       </c>
+      <c r="F21" s="7">
+        <v>7.6</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -6711,6 +6879,9 @@
       <c r="E22" s="7">
         <v>4.7</v>
       </c>
+      <c r="F22" s="7">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -6727,6 +6898,9 @@
       </c>
       <c r="E23" s="7">
         <v>6.4</v>
+      </c>
+      <c r="F23" s="7">
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -6759,6 +6933,9 @@
       <c r="D1" s="3">
         <v>3</v>
       </c>
+      <c r="E1" s="3">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6773,6 +6950,9 @@
       <c r="D2" s="7">
         <v>28.5</v>
       </c>
+      <c r="E2" s="7">
+        <v>28.6</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -6787,6 +6967,9 @@
       <c r="D3" s="7">
         <v>23.9</v>
       </c>
+      <c r="E3" s="7">
+        <v>24.2</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -6801,6 +6984,9 @@
       <c r="D4" s="7">
         <v>28.8</v>
       </c>
+      <c r="E4" s="7">
+        <v>29.1</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -6815,6 +7001,9 @@
       <c r="D5" s="7">
         <v>29.9</v>
       </c>
+      <c r="E5" s="7">
+        <v>30.2</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -6829,6 +7018,9 @@
       <c r="D6" s="7">
         <v>13.2</v>
       </c>
+      <c r="E6" s="7">
+        <v>13.8</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -6843,6 +7035,9 @@
       <c r="D7" s="7">
         <v>7.5</v>
       </c>
+      <c r="E7" s="7">
+        <v>8.1</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -6857,6 +7052,9 @@
       <c r="D8" s="7">
         <v>8.6</v>
       </c>
+      <c r="E8" s="7">
+        <v>9.2</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -6871,6 +7069,9 @@
       <c r="D9" s="7">
         <v>9.1</v>
       </c>
+      <c r="E9" s="7">
+        <v>8.6</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -6885,6 +7086,9 @@
       <c r="D10" s="7">
         <v>13.7</v>
       </c>
+      <c r="E10" s="7">
+        <v>14.3</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -6899,6 +7103,9 @@
       <c r="D11" s="7">
         <v>5.4</v>
       </c>
+      <c r="E11" s="7">
+        <v>5.6</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -6912,6 +7119,9 @@
       </c>
       <c r="D12" s="7">
         <v>5.2</v>
+      </c>
+      <c r="E12" s="7">
+        <v>5.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Data correction from app, race 3
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="13" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="15" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -6560,7 +6560,7 @@
         <v>28.1</v>
       </c>
       <c r="F6" s="7">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -6880,7 +6880,7 @@
         <v>4.7</v>
       </c>
       <c r="F22" s="7">
-        <v>4.5</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -7070,7 +7070,7 @@
         <v>9.1</v>
       </c>
       <c r="E9" s="7">
-        <v>8.6</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="10" spans="1:2">
@@ -7121,7 +7121,7 @@
         <v>5.2</v>
       </c>
       <c r="E12" s="7">
-        <v>5.4</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated race stats for Miami
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="15" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="12" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -175,6 +175,9 @@
   </si>
   <si>
     <t>AUD</t>
+  </si>
+  <si>
+    <t>-=16</t>
   </si>
 </sst>
 </file>
@@ -5769,6 +5772,9 @@
       <c r="F1" s="3">
         <v>4</v>
       </c>
+      <c r="G1" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5787,6 +5793,9 @@
         <v>24</v>
       </c>
       <c r="F2" s="2">
+        <v>54</v>
+      </c>
+      <c r="G2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5807,6 +5816,9 @@
         <v>43</v>
       </c>
       <c r="F3" s="2">
+        <v>41</v>
+      </c>
+      <c r="G3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5827,6 +5839,9 @@
         <v>27</v>
       </c>
       <c r="F4" s="2">
+        <v>42</v>
+      </c>
+      <c r="G4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5847,6 +5862,9 @@
         <v>50</v>
       </c>
       <c r="F5" s="2">
+        <v>42</v>
+      </c>
+      <c r="G5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5867,6 +5885,9 @@
         <v>13</v>
       </c>
       <c r="F6" s="2">
+        <v>52</v>
+      </c>
+      <c r="G6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5887,6 +5908,9 @@
         <v>5</v>
       </c>
       <c r="F7" s="2">
+        <v>-16</v>
+      </c>
+      <c r="G7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5907,6 +5931,9 @@
         <v>19</v>
       </c>
       <c r="F8" s="2">
+        <v>20</v>
+      </c>
+      <c r="G8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5927,6 +5954,9 @@
         <v>31</v>
       </c>
       <c r="F9" s="2">
+        <v>27</v>
+      </c>
+      <c r="G9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5947,6 +5977,9 @@
         <v>-1</v>
       </c>
       <c r="F10" s="2">
+        <v>20</v>
+      </c>
+      <c r="G10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5967,6 +6000,9 @@
         <v>4</v>
       </c>
       <c r="F11" s="2">
+        <v>19</v>
+      </c>
+      <c r="G11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5987,6 +6023,9 @@
         <v>10</v>
       </c>
       <c r="F12" s="2">
+        <v>-12</v>
+      </c>
+      <c r="G12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6007,6 +6046,9 @@
         <v>1</v>
       </c>
       <c r="F13" s="2">
+        <v>-4</v>
+      </c>
+      <c r="G13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6027,6 +6069,9 @@
         <v>4</v>
       </c>
       <c r="F14" s="2">
+        <v>20</v>
+      </c>
+      <c r="G14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6047,6 +6092,9 @@
         <v>-17</v>
       </c>
       <c r="F15" s="2">
+        <v>17</v>
+      </c>
+      <c r="G15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6067,6 +6115,9 @@
         <v>9</v>
       </c>
       <c r="F16" s="2">
+        <v>14</v>
+      </c>
+      <c r="G16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6087,6 +6138,9 @@
         <v>-14</v>
       </c>
       <c r="F17" s="2">
+        <v>6</v>
+      </c>
+      <c r="G17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6107,6 +6161,9 @@
         <v>10</v>
       </c>
       <c r="F18" s="2">
+        <v>-29</v>
+      </c>
+      <c r="G18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6127,6 +6184,9 @@
         <v>3</v>
       </c>
       <c r="F19" s="2">
+        <v>7</v>
+      </c>
+      <c r="G19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6147,6 +6207,9 @@
         <v>14</v>
       </c>
       <c r="F20" s="2">
+        <v>-8</v>
+      </c>
+      <c r="G20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6167,6 +6230,9 @@
         <v>4</v>
       </c>
       <c r="F21" s="2">
+        <v>13</v>
+      </c>
+      <c r="G21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6187,6 +6253,9 @@
         <v>2</v>
       </c>
       <c r="F22" s="2">
+        <v>4</v>
+      </c>
+      <c r="G22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6207,6 +6276,9 @@
         <v>4</v>
       </c>
       <c r="F23" s="2">
+        <v>19</v>
+      </c>
+      <c r="G23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6243,6 +6315,9 @@
       <c r="E1" s="3">
         <v>4</v>
       </c>
+      <c r="F1" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6258,6 +6333,9 @@
         <v>72</v>
       </c>
       <c r="E2" s="2">
+        <v>110</v>
+      </c>
+      <c r="F2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6275,6 +6353,9 @@
         <v>75</v>
       </c>
       <c r="E3" s="2">
+        <v>57</v>
+      </c>
+      <c r="F3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6292,6 +6373,9 @@
         <v>25</v>
       </c>
       <c r="E4" s="2">
+        <v>31</v>
+      </c>
+      <c r="F4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6309,6 +6393,9 @@
         <v>92</v>
       </c>
       <c r="E5" s="2">
+        <v>104</v>
+      </c>
+      <c r="F5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6326,6 +6413,9 @@
         <v>9</v>
       </c>
       <c r="E6" s="2">
+        <v>42</v>
+      </c>
+      <c r="F6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6343,6 +6433,9 @@
         <v>-4</v>
       </c>
       <c r="E7" s="2">
+        <v>23</v>
+      </c>
+      <c r="F7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6360,6 +6453,9 @@
         <v>18</v>
       </c>
       <c r="E8" s="2">
+        <v>2</v>
+      </c>
+      <c r="F8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6377,6 +6473,9 @@
         <v>23</v>
       </c>
       <c r="E9" s="2">
+        <v>-27</v>
+      </c>
+      <c r="F9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6394,6 +6493,9 @@
         <v>-12</v>
       </c>
       <c r="E10" s="2">
+        <v>38</v>
+      </c>
+      <c r="F10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6411,6 +6513,9 @@
         <v>25</v>
       </c>
       <c r="E11" s="2">
+        <v>17</v>
+      </c>
+      <c r="F11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6428,6 +6533,9 @@
         <v>5</v>
       </c>
       <c r="E12" s="2">
+        <v>24</v>
+      </c>
+      <c r="F12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6462,6 +6570,9 @@
       <c r="F1" s="3">
         <v>4</v>
       </c>
+      <c r="G1" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -6482,6 +6593,9 @@
       <c r="F2" s="6">
         <v>26.5</v>
       </c>
+      <c r="G2" s="1">
+        <v>26.4</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -6502,6 +6616,9 @@
       <c r="F3" s="7">
         <v>24.6</v>
       </c>
+      <c r="G3" s="1">
+        <v>24.7</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -6522,6 +6639,9 @@
       <c r="F4" s="7">
         <v>28.3</v>
       </c>
+      <c r="G4" s="1">
+        <v>28.6</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -6542,6 +6662,9 @@
       <c r="F5" s="7">
         <v>24.1</v>
       </c>
+      <c r="G5" s="1">
+        <v>24.4</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -6562,6 +6685,9 @@
       <c r="F6" s="7">
         <v>28.2</v>
       </c>
+      <c r="G6" s="1">
+        <v>28.3</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -6582,6 +6708,9 @@
       <c r="F7" s="7">
         <v>13.3</v>
       </c>
+      <c r="G7" s="1">
+        <v>12.7</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -6602,6 +6731,9 @@
       <c r="F8" s="6">
         <v>23.2</v>
       </c>
+      <c r="G8" s="1">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -6622,6 +6754,9 @@
       <c r="F9" s="7">
         <v>23.7</v>
       </c>
+      <c r="G9" s="1">
+        <v>24</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -6642,6 +6777,9 @@
       <c r="F10" s="6">
         <v>10.2</v>
       </c>
+      <c r="G10" s="1">
+        <v>9.6</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -6662,6 +6800,9 @@
       <c r="F11" s="7">
         <v>12.4</v>
       </c>
+      <c r="G11" s="1">
+        <v>13</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -6682,6 +6823,9 @@
       <c r="F12" s="6">
         <v>7.5</v>
       </c>
+      <c r="G12" s="1">
+        <v>8.1</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -6702,6 +6846,9 @@
       <c r="F13" s="7">
         <v>7.6</v>
       </c>
+      <c r="G13" s="1">
+        <v>7</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -6722,6 +6869,9 @@
       <c r="F14" s="7">
         <v>8.2</v>
       </c>
+      <c r="G14" s="1">
+        <v>8</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -6742,6 +6892,9 @@
       <c r="F15" s="7">
         <v>6.2</v>
       </c>
+      <c r="G15" s="1">
+        <v>5.6</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -6762,6 +6915,9 @@
       <c r="F16" s="7">
         <v>9.1</v>
       </c>
+      <c r="G16" s="1">
+        <v>9.7</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -6782,6 +6938,9 @@
       <c r="F17" s="7">
         <v>9.2</v>
       </c>
+      <c r="G17" s="1">
+        <v>9.4</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -6802,6 +6961,9 @@
       <c r="F18" s="7">
         <v>5</v>
       </c>
+      <c r="G18" s="1">
+        <v>4.4</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -6822,6 +6984,9 @@
       <c r="F19" s="7">
         <v>5.8</v>
       </c>
+      <c r="G19" s="1">
+        <v>5.2</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -6842,6 +7007,9 @@
       <c r="F20" s="6">
         <v>13</v>
       </c>
+      <c r="G20" s="1">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -6862,6 +7030,9 @@
       <c r="F21" s="7">
         <v>7.6</v>
       </c>
+      <c r="G21" s="1">
+        <v>8.2</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -6882,6 +7053,9 @@
       <c r="F22" s="7">
         <v>4.1</v>
       </c>
+      <c r="G22" s="1">
+        <v>3.9</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -6901,6 +7075,9 @@
       </c>
       <c r="F23" s="7">
         <v>7</v>
+      </c>
+      <c r="G23" s="1">
+        <v>7.6</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -6936,6 +7113,9 @@
       <c r="E1" s="3">
         <v>4</v>
       </c>
+      <c r="F1" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6953,6 +7133,9 @@
       <c r="E2" s="7">
         <v>28.6</v>
       </c>
+      <c r="F2" s="1">
+        <v>28.9</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -6970,6 +7153,9 @@
       <c r="E3" s="7">
         <v>24.2</v>
       </c>
+      <c r="F3" s="1">
+        <v>24.5</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -6987,6 +7173,9 @@
       <c r="E4" s="7">
         <v>29.1</v>
       </c>
+      <c r="F4" s="1">
+        <v>29.2</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -7004,6 +7193,9 @@
       <c r="E5" s="7">
         <v>30.2</v>
       </c>
+      <c r="F5" s="1">
+        <v>30.5</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -7021,6 +7213,9 @@
       <c r="E6" s="7">
         <v>13.8</v>
       </c>
+      <c r="F6" s="1">
+        <v>14.4</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -7038,6 +7233,9 @@
       <c r="E7" s="7">
         <v>8.1</v>
       </c>
+      <c r="F7" s="1">
+        <v>8.7</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -7055,6 +7253,9 @@
       <c r="E8" s="7">
         <v>9.2</v>
       </c>
+      <c r="F8" s="1">
+        <v>9.8</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -7072,6 +7273,9 @@
       <c r="E9" s="7">
         <v>8.5</v>
       </c>
+      <c r="F9" s="1">
+        <v>7.9</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -7089,6 +7293,9 @@
       <c r="E10" s="7">
         <v>14.3</v>
       </c>
+      <c r="F10" s="1">
+        <v>14.9</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -7106,6 +7313,9 @@
       <c r="E11" s="7">
         <v>5.6</v>
       </c>
+      <c r="F11" s="1">
+        <v>5</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -7122,6 +7332,9 @@
       </c>
       <c r="E12" s="7">
         <v>5</v>
+      </c>
+      <c r="F12" s="1">
+        <v>5.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated stats for race 6 Canada
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="12" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="15" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -5775,6 +5775,9 @@
       <c r="G1" s="3">
         <v>5</v>
       </c>
+      <c r="H1" s="3">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5796,6 +5799,9 @@
         <v>54</v>
       </c>
       <c r="G2" s="2">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5819,6 +5825,9 @@
         <v>41</v>
       </c>
       <c r="G3" s="2">
+        <v>12</v>
+      </c>
+      <c r="H3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5842,6 +5851,9 @@
         <v>42</v>
       </c>
       <c r="G4" s="2">
+        <v>4</v>
+      </c>
+      <c r="H4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5865,6 +5877,9 @@
         <v>42</v>
       </c>
       <c r="G5" s="2">
+        <v>62</v>
+      </c>
+      <c r="H5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5888,6 +5903,9 @@
         <v>52</v>
       </c>
       <c r="G6" s="2">
+        <v>26</v>
+      </c>
+      <c r="H6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5911,6 +5929,9 @@
         <v>-16</v>
       </c>
       <c r="G7" s="2">
+        <v>6</v>
+      </c>
+      <c r="H7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5934,6 +5955,9 @@
         <v>20</v>
       </c>
       <c r="G8" s="2">
+        <v>42</v>
+      </c>
+      <c r="H8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5957,6 +5981,9 @@
         <v>27</v>
       </c>
       <c r="G9" s="2">
+        <v>27</v>
+      </c>
+      <c r="H9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5980,6 +6007,9 @@
         <v>20</v>
       </c>
       <c r="G10" s="2">
+        <v>-8</v>
+      </c>
+      <c r="H10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6003,6 +6033,9 @@
         <v>19</v>
       </c>
       <c r="G11" s="2">
+        <v>11</v>
+      </c>
+      <c r="H11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6026,6 +6059,9 @@
         <v>-12</v>
       </c>
       <c r="G12" s="2">
+        <v>23</v>
+      </c>
+      <c r="H12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6049,6 +6085,9 @@
         <v>-4</v>
       </c>
       <c r="G13" s="2">
+        <v>-16</v>
+      </c>
+      <c r="H13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6072,6 +6111,9 @@
         <v>20</v>
       </c>
       <c r="G14" s="2">
+        <v>-26</v>
+      </c>
+      <c r="H14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6095,6 +6137,9 @@
         <v>17</v>
       </c>
       <c r="G15" s="2">
+        <v>11</v>
+      </c>
+      <c r="H15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6118,6 +6163,9 @@
         <v>14</v>
       </c>
       <c r="G16" s="2">
+        <v>8</v>
+      </c>
+      <c r="H16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6141,6 +6189,9 @@
         <v>6</v>
       </c>
       <c r="G17" s="2">
+        <v>10</v>
+      </c>
+      <c r="H17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6164,6 +6215,9 @@
         <v>-29</v>
       </c>
       <c r="G18" s="2">
+        <v>1</v>
+      </c>
+      <c r="H18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6187,6 +6241,9 @@
         <v>7</v>
       </c>
       <c r="G19" s="2">
+        <v>5</v>
+      </c>
+      <c r="H19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6210,6 +6267,9 @@
         <v>-8</v>
       </c>
       <c r="G20" s="2">
+        <v>16</v>
+      </c>
+      <c r="H20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6233,6 +6293,9 @@
         <v>13</v>
       </c>
       <c r="G21" s="2">
+        <v>25</v>
+      </c>
+      <c r="H21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6256,6 +6319,9 @@
         <v>4</v>
       </c>
       <c r="G22" s="2">
+        <v>12</v>
+      </c>
+      <c r="H22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6279,6 +6345,9 @@
         <v>19</v>
       </c>
       <c r="G23" s="2">
+        <v>-11</v>
+      </c>
+      <c r="H23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6318,6 +6387,9 @@
       <c r="F1" s="3">
         <v>5</v>
       </c>
+      <c r="G1" s="3">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6336,6 +6408,9 @@
         <v>110</v>
       </c>
       <c r="F2" s="2">
+        <v>33</v>
+      </c>
+      <c r="G2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6356,6 +6431,9 @@
         <v>57</v>
       </c>
       <c r="F3" s="2">
+        <v>69</v>
+      </c>
+      <c r="G3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6376,6 +6454,9 @@
         <v>31</v>
       </c>
       <c r="F4" s="2">
+        <v>44</v>
+      </c>
+      <c r="G4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6396,6 +6477,9 @@
         <v>104</v>
       </c>
       <c r="F5" s="2">
+        <v>76</v>
+      </c>
+      <c r="G5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6416,6 +6500,9 @@
         <v>42</v>
       </c>
       <c r="F6" s="2">
+        <v>6</v>
+      </c>
+      <c r="G6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6436,6 +6523,9 @@
         <v>23</v>
       </c>
       <c r="F7" s="2">
+        <v>19</v>
+      </c>
+      <c r="G7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6456,6 +6546,9 @@
         <v>2</v>
       </c>
       <c r="F8" s="2">
+        <v>22</v>
+      </c>
+      <c r="G8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6476,6 +6569,9 @@
         <v>-27</v>
       </c>
       <c r="F9" s="2">
+        <v>11</v>
+      </c>
+      <c r="G9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6496,6 +6592,9 @@
         <v>38</v>
       </c>
       <c r="F10" s="2">
+        <v>-14</v>
+      </c>
+      <c r="G10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6516,6 +6615,9 @@
         <v>17</v>
       </c>
       <c r="F11" s="2">
+        <v>46</v>
+      </c>
+      <c r="G11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6536,6 +6638,9 @@
         <v>24</v>
       </c>
       <c r="F12" s="2">
+        <v>2</v>
+      </c>
+      <c r="G12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6573,6 +6678,9 @@
       <c r="G1" s="3">
         <v>5</v>
       </c>
+      <c r="H1" s="3">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -6596,6 +6704,9 @@
       <c r="G2" s="1">
         <v>26.4</v>
       </c>
+      <c r="H2" s="1">
+        <v>26.5</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -6619,6 +6730,9 @@
       <c r="G3" s="1">
         <v>24.7</v>
       </c>
+      <c r="H3" s="1">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -6642,6 +6756,9 @@
       <c r="G4" s="1">
         <v>28.6</v>
       </c>
+      <c r="H4" s="1">
+        <v>28.5</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -6665,6 +6782,9 @@
       <c r="G5" s="1">
         <v>24.4</v>
       </c>
+      <c r="H5" s="1">
+        <v>24.7</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -6688,6 +6808,9 @@
       <c r="G6" s="1">
         <v>28.3</v>
       </c>
+      <c r="H6" s="1">
+        <v>28.4</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -6711,6 +6834,9 @@
       <c r="G7" s="1">
         <v>12.7</v>
       </c>
+      <c r="H7" s="1">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -6734,6 +6860,9 @@
       <c r="G8" s="1">
         <v>23.5</v>
       </c>
+      <c r="H8" s="1">
+        <v>23.6</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -6757,6 +6886,9 @@
       <c r="G9" s="1">
         <v>24</v>
       </c>
+      <c r="H9" s="1">
+        <v>24.1</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -6780,6 +6912,9 @@
       <c r="G10" s="1">
         <v>9.6</v>
       </c>
+      <c r="H10" s="1">
+        <v>9</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -6803,6 +6938,9 @@
       <c r="G11" s="1">
         <v>13</v>
       </c>
+      <c r="H11" s="1">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -6826,6 +6964,9 @@
       <c r="G12" s="1">
         <v>8.1</v>
       </c>
+      <c r="H12" s="1">
+        <v>7.9</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -6849,6 +6990,9 @@
       <c r="G13" s="1">
         <v>7</v>
       </c>
+      <c r="H13" s="1">
+        <v>6.4</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -6872,6 +7016,9 @@
       <c r="G14" s="1">
         <v>8</v>
       </c>
+      <c r="H14" s="1">
+        <v>7.4</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -6895,6 +7042,9 @@
       <c r="G15" s="1">
         <v>5.6</v>
       </c>
+      <c r="H15" s="1">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -6918,6 +7068,9 @@
       <c r="G16" s="1">
         <v>9.7</v>
       </c>
+      <c r="H16" s="1">
+        <v>9.9</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -6941,6 +7094,9 @@
       <c r="G17" s="1">
         <v>9.4</v>
       </c>
+      <c r="H17" s="1">
+        <v>8.8</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -6964,6 +7120,9 @@
       <c r="G18" s="1">
         <v>4.4</v>
       </c>
+      <c r="H18" s="1">
+        <v>3.8</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -6987,6 +7146,9 @@
       <c r="G19" s="1">
         <v>5.2</v>
       </c>
+      <c r="H19" s="1">
+        <v>5.4</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -7010,6 +7172,9 @@
       <c r="G20" s="1">
         <v>12.8</v>
       </c>
+      <c r="H20" s="1">
+        <v>12.2</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -7033,6 +7198,9 @@
       <c r="G21" s="1">
         <v>8.2</v>
       </c>
+      <c r="H21" s="1">
+        <v>8.8</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -7056,6 +7224,9 @@
       <c r="G22" s="1">
         <v>3.9</v>
       </c>
+      <c r="H22" s="1">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -7078,6 +7249,9 @@
       </c>
       <c r="G23" s="1">
         <v>7.6</v>
+      </c>
+      <c r="H23" s="1">
+        <v>7</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -7116,6 +7290,9 @@
       <c r="F1" s="3">
         <v>5</v>
       </c>
+      <c r="G1" s="3">
+        <v>6</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -7136,6 +7313,9 @@
       <c r="F2" s="1">
         <v>28.9</v>
       </c>
+      <c r="G2" s="1">
+        <v>29.2</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -7156,6 +7336,9 @@
       <c r="F3" s="1">
         <v>24.5</v>
       </c>
+      <c r="G3" s="1">
+        <v>24.8</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -7176,6 +7359,9 @@
       <c r="F4" s="1">
         <v>29.2</v>
       </c>
+      <c r="G4" s="1">
+        <v>29.3</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -7196,6 +7382,9 @@
       <c r="F5" s="1">
         <v>30.5</v>
       </c>
+      <c r="G5" s="1">
+        <v>30.8</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -7216,6 +7405,9 @@
       <c r="F6" s="1">
         <v>14.4</v>
       </c>
+      <c r="G6" s="1">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -7236,6 +7428,9 @@
       <c r="F7" s="1">
         <v>8.7</v>
       </c>
+      <c r="G7" s="1">
+        <v>9.3</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -7256,6 +7451,9 @@
       <c r="F8" s="1">
         <v>9.8</v>
       </c>
+      <c r="G8" s="1">
+        <v>10.4</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -7276,6 +7474,9 @@
       <c r="F9" s="1">
         <v>7.9</v>
       </c>
+      <c r="G9" s="1">
+        <v>7.3</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -7296,6 +7497,9 @@
       <c r="F10" s="1">
         <v>14.9</v>
       </c>
+      <c r="G10" s="1">
+        <v>15.5</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -7316,6 +7520,9 @@
       <c r="F11" s="1">
         <v>5</v>
       </c>
+      <c r="G11" s="1">
+        <v>4.4</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -7335,6 +7542,9 @@
       </c>
       <c r="F12" s="1">
         <v>5.6</v>
+      </c>
+      <c r="G12" s="1">
+        <v>6.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monaco corrections, Barcelona updates, Austria team selection
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -181,6 +181,9 @@
   </si>
   <si>
     <t>0-11</t>
+  </si>
+  <si>
+    <t>3.53.2</t>
   </si>
 </sst>
 </file>
@@ -5784,6 +5787,9 @@
       <c r="I1" s="3">
         <v>7</v>
       </c>
+      <c r="J1" s="3">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5811,6 +5817,9 @@
         <v>-17</v>
       </c>
       <c r="I2" s="2">
+        <v>23</v>
+      </c>
+      <c r="J2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5837,9 +5846,12 @@
         <v>12</v>
       </c>
       <c r="H3" s="2">
+        <v>16</v>
+      </c>
+      <c r="I3" s="2">
         <v>19</v>
       </c>
-      <c r="I3" s="2">
+      <c r="J3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5869,6 +5881,9 @@
         <v>0</v>
       </c>
       <c r="I4" s="2">
+        <v>28</v>
+      </c>
+      <c r="J4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5898,6 +5913,9 @@
         <v>55</v>
       </c>
       <c r="I5" s="2">
+        <v>-4</v>
+      </c>
+      <c r="J5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5927,6 +5945,9 @@
         <v>-11</v>
       </c>
       <c r="I6" s="2">
+        <v>22</v>
+      </c>
+      <c r="J6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5953,9 +5974,12 @@
         <v>6</v>
       </c>
       <c r="H7" s="2">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="I7" s="2">
+        <v>22</v>
+      </c>
+      <c r="J7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5985,6 +6009,9 @@
         <v>27</v>
       </c>
       <c r="I8" s="2">
+        <v>56</v>
+      </c>
+      <c r="J8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6016,6 +6043,9 @@
       <c r="I9" s="2">
         <v>0</v>
       </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="2" t="s">
@@ -6043,6 +6073,9 @@
         <v>9</v>
       </c>
       <c r="I10" s="2">
+        <v>-16</v>
+      </c>
+      <c r="J10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6072,6 +6105,9 @@
         <v>-3</v>
       </c>
       <c r="I11" s="2">
+        <v>11</v>
+      </c>
+      <c r="J11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6098,9 +6134,12 @@
         <v>23</v>
       </c>
       <c r="H12" s="2">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="I12" s="2">
+        <v>9</v>
+      </c>
+      <c r="J12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6127,9 +6166,12 @@
         <v>-16</v>
       </c>
       <c r="H13" s="2">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="I13" s="2">
+        <v>10</v>
+      </c>
+      <c r="J13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6159,6 +6201,9 @@
         <v>15</v>
       </c>
       <c r="I14" s="2">
+        <v>-17</v>
+      </c>
+      <c r="J14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6188,6 +6233,9 @@
         <v>-20</v>
       </c>
       <c r="I15" s="2">
+        <v>-20</v>
+      </c>
+      <c r="J15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6217,6 +6265,9 @@
         <v>12</v>
       </c>
       <c r="I16" s="2">
+        <v>8</v>
+      </c>
+      <c r="J16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6246,6 +6297,9 @@
         <v>-19</v>
       </c>
       <c r="I17" s="2">
+        <v>7</v>
+      </c>
+      <c r="J17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6275,6 +6329,9 @@
         <v>3</v>
       </c>
       <c r="I18" s="2">
+        <v>-15</v>
+      </c>
+      <c r="J18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6304,6 +6361,9 @@
         <v>5</v>
       </c>
       <c r="I19" s="2">
+        <v>7</v>
+      </c>
+      <c r="J19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6330,9 +6390,12 @@
         <v>16</v>
       </c>
       <c r="H20" s="2">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="I20" s="2">
+        <v>17</v>
+      </c>
+      <c r="J20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6362,6 +6425,9 @@
         <v>0</v>
       </c>
       <c r="I21" s="2">
+        <v>9</v>
+      </c>
+      <c r="J21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6391,6 +6457,9 @@
         <v>-20</v>
       </c>
       <c r="I22" s="2">
+        <v>-18</v>
+      </c>
+      <c r="J22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6420,6 +6489,9 @@
         <v>8</v>
       </c>
       <c r="I23" s="2">
+        <v>8</v>
+      </c>
+      <c r="J23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6465,6 +6537,9 @@
       <c r="H1" s="3">
         <v>7</v>
       </c>
+      <c r="I1" s="3">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6486,9 +6561,12 @@
         <v>33</v>
       </c>
       <c r="G2" s="2">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H2" s="2">
+        <v>67</v>
+      </c>
+      <c r="I2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6515,6 +6593,9 @@
         <v>29</v>
       </c>
       <c r="H3" s="2">
+        <v>58</v>
+      </c>
+      <c r="I3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6538,9 +6619,12 @@
         <v>44</v>
       </c>
       <c r="G4" s="2">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H4" s="2">
+        <v>59</v>
+      </c>
+      <c r="I4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6567,6 +6651,9 @@
         <v>70</v>
       </c>
       <c r="H5" s="2">
+        <v>39</v>
+      </c>
+      <c r="I5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6593,6 +6680,9 @@
         <v>9</v>
       </c>
       <c r="H6" s="2">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6619,6 +6709,9 @@
         <v>-8</v>
       </c>
       <c r="H7" s="2">
+        <v>16</v>
+      </c>
+      <c r="I7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6642,9 +6735,12 @@
         <v>22</v>
       </c>
       <c r="G8" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="H8" s="2">
+        <v>26</v>
+      </c>
+      <c r="I8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6671,6 +6767,9 @@
         <v>21</v>
       </c>
       <c r="H9" s="2">
+        <v>2</v>
+      </c>
+      <c r="I9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6697,6 +6796,9 @@
         <v>-4</v>
       </c>
       <c r="H10" s="2">
+        <v>-36</v>
+      </c>
+      <c r="I10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6720,9 +6822,12 @@
         <v>46</v>
       </c>
       <c r="G11" s="2">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="H11" s="2">
+        <v>31</v>
+      </c>
+      <c r="I11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6749,6 +6854,9 @@
         <v>-13</v>
       </c>
       <c r="H12" s="2">
+        <v>-9</v>
+      </c>
+      <c r="I12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6792,6 +6900,9 @@
       <c r="I1" s="3">
         <v>7</v>
       </c>
+      <c r="J1" s="3">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -6821,6 +6932,9 @@
       <c r="I2" s="1">
         <v>26.2</v>
       </c>
+      <c r="J2" s="1">
+        <v>25.9</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -6850,6 +6964,9 @@
       <c r="I3" s="1">
         <v>25.1</v>
       </c>
+      <c r="J3" s="1">
+        <v>25</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -6879,6 +6996,9 @@
       <c r="I4" s="1">
         <v>28.2</v>
       </c>
+      <c r="J4" s="1">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -6908,6 +7028,9 @@
       <c r="I5" s="1">
         <v>25</v>
       </c>
+      <c r="J5" s="1">
+        <v>25.3</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -6937,6 +7060,9 @@
       <c r="I6" s="1">
         <v>28.3</v>
       </c>
+      <c r="J6" s="1">
+        <v>28</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -6966,6 +7092,9 @@
       <c r="I7" s="1">
         <v>11.5</v>
       </c>
+      <c r="J7" s="1">
+        <v>12.1</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -6995,6 +7124,9 @@
       <c r="I8" s="1">
         <v>23.9</v>
       </c>
+      <c r="J8" s="1">
+        <v>24.2</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -7024,6 +7156,9 @@
       <c r="I9" s="1">
         <v>23.8</v>
       </c>
+      <c r="J9" s="1">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -7053,6 +7188,9 @@
       <c r="I10" s="1">
         <v>8.8</v>
       </c>
+      <c r="J10" s="1">
+        <v>8.2</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -7082,6 +7220,9 @@
       <c r="I11" s="1">
         <v>12.6</v>
       </c>
+      <c r="J11" s="1">
+        <v>12</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -7111,6 +7252,9 @@
       <c r="I12" s="1">
         <v>8.1</v>
       </c>
+      <c r="J12" s="1">
+        <v>8.7</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -7140,6 +7284,9 @@
       <c r="I13" s="1">
         <v>5.8</v>
       </c>
+      <c r="J13" s="1">
+        <v>5.6</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -7169,6 +7316,9 @@
       <c r="I14" s="1">
         <v>6.8</v>
       </c>
+      <c r="J14" s="1">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -7198,6 +7348,9 @@
       <c r="I15" s="1">
         <v>4.8</v>
       </c>
+      <c r="J15" s="1">
+        <v>4.2</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -7227,6 +7380,9 @@
       <c r="I16" s="1">
         <v>10.1</v>
       </c>
+      <c r="J16" s="1">
+        <v>10.3</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -7256,6 +7412,9 @@
       <c r="I17" s="1">
         <v>8.2</v>
       </c>
+      <c r="J17" s="1">
+        <v>7.6</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -7283,7 +7442,10 @@
         <v>3.8</v>
       </c>
       <c r="I18" s="1">
-        <v>3.5</v>
+        <v>3.2</v>
+      </c>
+      <c r="J18" s="1">
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -7314,6 +7476,9 @@
       <c r="I19" s="1">
         <v>5.6</v>
       </c>
+      <c r="J19" s="1">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -7343,6 +7508,9 @@
       <c r="I20" s="1">
         <v>11.6</v>
       </c>
+      <c r="J20" s="1">
+        <v>12.2</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -7372,6 +7540,9 @@
       <c r="I21" s="1">
         <v>9.4</v>
       </c>
+      <c r="J21" s="1">
+        <v>10</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -7401,6 +7572,9 @@
       <c r="I22" s="1">
         <v>3.9</v>
       </c>
+      <c r="J22" s="1">
+        <v>3.3</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -7429,6 +7603,9 @@
       </c>
       <c r="I23" s="1">
         <v>6.8</v>
+      </c>
+      <c r="J23" s="1">
+        <v>6.2</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -7473,6 +7650,9 @@
       <c r="H1" s="3">
         <v>7</v>
       </c>
+      <c r="I1" s="3">
+        <v>8</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -7499,6 +7679,9 @@
       <c r="H2" s="1">
         <v>29.5</v>
       </c>
+      <c r="I2" s="1">
+        <v>29.8</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -7525,6 +7708,9 @@
       <c r="H3" s="1">
         <v>25.1</v>
       </c>
+      <c r="I3" s="1">
+        <v>25.4</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -7551,6 +7737,9 @@
       <c r="H4" s="1">
         <v>29.4</v>
       </c>
+      <c r="I4" s="1">
+        <v>29.7</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -7577,6 +7766,9 @@
       <c r="H5" s="1">
         <v>31.1</v>
       </c>
+      <c r="I5" s="1">
+        <v>31.4</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -7603,6 +7795,9 @@
       <c r="H6" s="1">
         <v>15.6</v>
       </c>
+      <c r="I6" s="1">
+        <v>15</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -7629,6 +7824,9 @@
       <c r="H7" s="1">
         <v>9.9</v>
       </c>
+      <c r="I7" s="1">
+        <v>10.5</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -7655,6 +7853,9 @@
       <c r="H8" s="1">
         <v>10.6</v>
       </c>
+      <c r="I8" s="1">
+        <v>10.4</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -7681,6 +7882,9 @@
       <c r="H9" s="1">
         <v>7.5</v>
       </c>
+      <c r="I9" s="1">
+        <v>6.9</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -7707,6 +7911,9 @@
       <c r="H10" s="1">
         <v>16.1</v>
       </c>
+      <c r="I10" s="1">
+        <v>16.7</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -7733,6 +7940,9 @@
       <c r="H11" s="1">
         <v>3.8</v>
       </c>
+      <c r="I11" s="1">
+        <v>4.4</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -7758,6 +7968,9 @@
       </c>
       <c r="H12" s="1">
         <v>6</v>
+      </c>
+      <c r="I12" s="1">
+        <v>5.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated predict and data for Silverstone
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -5790,6 +5790,9 @@
       <c r="J1" s="3">
         <v>8</v>
       </c>
+      <c r="K1" s="3">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5820,6 +5823,9 @@
         <v>23</v>
       </c>
       <c r="J2" s="2">
+        <v>11</v>
+      </c>
+      <c r="K2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5852,6 +5858,9 @@
         <v>19</v>
       </c>
       <c r="J3" s="2">
+        <v>23</v>
+      </c>
+      <c r="K3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5884,6 +5893,9 @@
         <v>28</v>
       </c>
       <c r="J4" s="2">
+        <v>35</v>
+      </c>
+      <c r="K4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5916,6 +5928,9 @@
         <v>-4</v>
       </c>
       <c r="J5" s="2">
+        <v>35</v>
+      </c>
+      <c r="K5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5948,6 +5963,9 @@
         <v>22</v>
       </c>
       <c r="J6" s="2">
+        <v>43</v>
+      </c>
+      <c r="K6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5980,6 +5998,9 @@
         <v>22</v>
       </c>
       <c r="J7" s="2">
+        <v>15</v>
+      </c>
+      <c r="K7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6012,6 +6033,9 @@
         <v>56</v>
       </c>
       <c r="J8" s="2">
+        <v>27</v>
+      </c>
+      <c r="K8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6044,6 +6068,9 @@
         <v>0</v>
       </c>
       <c r="J9" s="2">
+        <v>9</v>
+      </c>
+      <c r="K9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6076,6 +6103,9 @@
         <v>-16</v>
       </c>
       <c r="J10" s="2">
+        <v>7</v>
+      </c>
+      <c r="K10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6108,6 +6138,9 @@
         <v>11</v>
       </c>
       <c r="J11" s="2">
+        <v>-17</v>
+      </c>
+      <c r="K11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6140,6 +6173,9 @@
         <v>9</v>
       </c>
       <c r="J12" s="2">
+        <v>7</v>
+      </c>
+      <c r="K12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6172,6 +6208,9 @@
         <v>10</v>
       </c>
       <c r="J13" s="2">
+        <v>6</v>
+      </c>
+      <c r="K13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6204,6 +6243,9 @@
         <v>-17</v>
       </c>
       <c r="J14" s="2">
+        <v>7</v>
+      </c>
+      <c r="K14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6236,6 +6278,9 @@
         <v>-20</v>
       </c>
       <c r="J15" s="2">
+        <v>-17</v>
+      </c>
+      <c r="K15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6268,6 +6313,9 @@
         <v>8</v>
       </c>
       <c r="J16" s="2">
+        <v>7</v>
+      </c>
+      <c r="K16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6300,6 +6348,9 @@
         <v>7</v>
       </c>
       <c r="J17" s="2">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6332,6 +6383,9 @@
         <v>-15</v>
       </c>
       <c r="J18" s="2">
+        <v>5</v>
+      </c>
+      <c r="K18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6364,6 +6418,9 @@
         <v>7</v>
       </c>
       <c r="J19" s="2">
+        <v>5</v>
+      </c>
+      <c r="K19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6396,6 +6453,9 @@
         <v>17</v>
       </c>
       <c r="J20" s="2">
+        <v>3</v>
+      </c>
+      <c r="K20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6428,6 +6488,9 @@
         <v>9</v>
       </c>
       <c r="J21" s="2">
+        <v>10</v>
+      </c>
+      <c r="K21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6460,6 +6523,9 @@
         <v>-18</v>
       </c>
       <c r="J22" s="2">
+        <v>-17</v>
+      </c>
+      <c r="K22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6492,6 +6558,9 @@
         <v>8</v>
       </c>
       <c r="J23" s="2">
+        <v>-17</v>
+      </c>
+      <c r="K23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6540,6 +6609,9 @@
       <c r="I1" s="3">
         <v>8</v>
       </c>
+      <c r="J1" s="3">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6567,6 +6639,9 @@
         <v>67</v>
       </c>
       <c r="I2" s="2">
+        <v>49</v>
+      </c>
+      <c r="J2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6596,6 +6671,9 @@
         <v>58</v>
       </c>
       <c r="I3" s="2">
+        <v>56</v>
+      </c>
+      <c r="J3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6625,6 +6703,9 @@
         <v>59</v>
       </c>
       <c r="I4" s="2">
+        <v>68</v>
+      </c>
+      <c r="J4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6654,6 +6735,9 @@
         <v>39</v>
       </c>
       <c r="I5" s="2">
+        <v>85</v>
+      </c>
+      <c r="J5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6683,6 +6767,9 @@
         <v>1</v>
       </c>
       <c r="I6" s="2">
+        <v>-6</v>
+      </c>
+      <c r="J6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6712,6 +6799,9 @@
         <v>16</v>
       </c>
       <c r="I7" s="2">
+        <v>13</v>
+      </c>
+      <c r="J7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6741,6 +6831,9 @@
         <v>26</v>
       </c>
       <c r="I8" s="2">
+        <v>38</v>
+      </c>
+      <c r="J8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6770,6 +6863,9 @@
         <v>2</v>
       </c>
       <c r="I9" s="2">
+        <v>15</v>
+      </c>
+      <c r="J9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6799,6 +6895,9 @@
         <v>-36</v>
       </c>
       <c r="I10" s="2">
+        <v>-11</v>
+      </c>
+      <c r="J10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6828,6 +6927,9 @@
         <v>31</v>
       </c>
       <c r="I11" s="2">
+        <v>21</v>
+      </c>
+      <c r="J11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6857,6 +6959,9 @@
         <v>-9</v>
       </c>
       <c r="I12" s="2">
+        <v>-35</v>
+      </c>
+      <c r="J12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6903,6 +7008,9 @@
       <c r="J1" s="3">
         <v>8</v>
       </c>
+      <c r="K1" s="3">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -6935,6 +7043,9 @@
       <c r="J2" s="1">
         <v>25.9</v>
       </c>
+      <c r="K2" s="1">
+        <v>25.6</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -6967,6 +7078,9 @@
       <c r="J3" s="1">
         <v>25</v>
       </c>
+      <c r="K3" s="1">
+        <v>24.9</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -6999,6 +7113,9 @@
       <c r="J4" s="1">
         <v>27.9</v>
       </c>
+      <c r="K4" s="1">
+        <v>27.8</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -7031,6 +7148,9 @@
       <c r="J5" s="1">
         <v>25.3</v>
       </c>
+      <c r="K5" s="1">
+        <v>25.4</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -7063,6 +7183,9 @@
       <c r="J6" s="1">
         <v>28</v>
       </c>
+      <c r="K6" s="1">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -7095,6 +7218,9 @@
       <c r="J7" s="1">
         <v>12.1</v>
       </c>
+      <c r="K7" s="1">
+        <v>12.7</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -7127,6 +7253,9 @@
       <c r="J8" s="1">
         <v>24.2</v>
       </c>
+      <c r="K8" s="1">
+        <v>24.5</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -7159,6 +7288,9 @@
       <c r="J9" s="1">
         <v>23.5</v>
       </c>
+      <c r="K9" s="1">
+        <v>23.2</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -7191,6 +7323,9 @@
       <c r="J10" s="1">
         <v>8.2</v>
       </c>
+      <c r="K10" s="1">
+        <v>7.6</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -7223,6 +7358,9 @@
       <c r="J11" s="1">
         <v>12</v>
       </c>
+      <c r="K11" s="1">
+        <v>11.4</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -7255,6 +7393,9 @@
       <c r="J12" s="1">
         <v>8.7</v>
       </c>
+      <c r="K12" s="1">
+        <v>8.9</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -7287,6 +7428,9 @@
       <c r="J13" s="1">
         <v>5.6</v>
       </c>
+      <c r="K13" s="1">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -7319,6 +7463,9 @@
       <c r="J14" s="1">
         <v>6.2</v>
       </c>
+      <c r="K14" s="1">
+        <v>5.6</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -7351,6 +7498,9 @@
       <c r="J15" s="1">
         <v>4.2</v>
       </c>
+      <c r="K15" s="1">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -7383,6 +7533,9 @@
       <c r="J16" s="1">
         <v>10.3</v>
       </c>
+      <c r="K16" s="1">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -7415,6 +7568,9 @@
       <c r="J17" s="1">
         <v>7.6</v>
       </c>
+      <c r="K17" s="1">
+        <v>7</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -7447,6 +7603,9 @@
       <c r="J18" s="1">
         <v>3</v>
       </c>
+      <c r="K18" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -7479,6 +7638,9 @@
       <c r="J19" s="1">
         <v>5.8</v>
       </c>
+      <c r="K19" s="1">
+        <v>6</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -7511,6 +7673,9 @@
       <c r="J20" s="1">
         <v>12.2</v>
       </c>
+      <c r="K20" s="1">
+        <v>12.8</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -7543,6 +7708,9 @@
       <c r="J21" s="1">
         <v>10</v>
       </c>
+      <c r="K21" s="1">
+        <v>9.8</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -7575,6 +7743,9 @@
       <c r="J22" s="1">
         <v>3.3</v>
       </c>
+      <c r="K22" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -7606,6 +7777,9 @@
       </c>
       <c r="J23" s="1">
         <v>6.2</v>
+      </c>
+      <c r="K23" s="1">
+        <v>5.6</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -7653,6 +7827,9 @@
       <c r="I1" s="3">
         <v>8</v>
       </c>
+      <c r="J1" s="3">
+        <v>9</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -7682,6 +7859,9 @@
       <c r="I2" s="1">
         <v>29.8</v>
       </c>
+      <c r="J2" s="1">
+        <v>30.1</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -7711,6 +7891,9 @@
       <c r="I3" s="1">
         <v>25.4</v>
       </c>
+      <c r="J3" s="1">
+        <v>25.7</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -7740,6 +7923,9 @@
       <c r="I4" s="1">
         <v>29.7</v>
       </c>
+      <c r="J4" s="1">
+        <v>30</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -7769,6 +7955,9 @@
       <c r="I5" s="1">
         <v>31.4</v>
       </c>
+      <c r="J5" s="1">
+        <v>31.7</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -7798,6 +7987,9 @@
       <c r="I6" s="1">
         <v>15</v>
       </c>
+      <c r="J6" s="1">
+        <v>14.4</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -7827,6 +8019,9 @@
       <c r="I7" s="1">
         <v>10.5</v>
       </c>
+      <c r="J7" s="1">
+        <v>11.1</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -7856,6 +8051,9 @@
       <c r="I8" s="1">
         <v>10.4</v>
       </c>
+      <c r="J8" s="1">
+        <v>10.2</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -7885,6 +8083,9 @@
       <c r="I9" s="1">
         <v>6.9</v>
       </c>
+      <c r="J9" s="1">
+        <v>6.3</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -7914,6 +8115,9 @@
       <c r="I10" s="1">
         <v>16.7</v>
       </c>
+      <c r="J10" s="1">
+        <v>17.3</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -7943,6 +8147,9 @@
       <c r="I11" s="1">
         <v>4.4</v>
       </c>
+      <c r="J11" s="1">
+        <v>5</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -7971,6 +8178,9 @@
       </c>
       <c r="I12" s="1">
         <v>5.4</v>
+      </c>
+      <c r="J12" s="1">
+        <v>4.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated race data after Hungary
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="13" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="12" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -5799,6 +5799,9 @@
       <c r="M1" s="3">
         <v>11</v>
       </c>
+      <c r="N1" s="3">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5838,6 +5841,9 @@
         <v>40</v>
       </c>
       <c r="M2" s="2">
+        <v>37</v>
+      </c>
+      <c r="N2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5879,6 +5885,9 @@
         <v>19</v>
       </c>
       <c r="M3" s="2">
+        <v>-11</v>
+      </c>
+      <c r="N3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5920,6 +5929,9 @@
         <v>-11</v>
       </c>
       <c r="M4" s="2">
+        <v>23</v>
+      </c>
+      <c r="N4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5961,6 +5973,9 @@
         <v>38</v>
       </c>
       <c r="M5" s="2">
+        <v>28</v>
+      </c>
+      <c r="N5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6002,6 +6017,9 @@
         <v>26</v>
       </c>
       <c r="M6" s="2">
+        <v>39</v>
+      </c>
+      <c r="N6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6043,6 +6061,9 @@
         <v>38</v>
       </c>
       <c r="M7" s="2">
+        <v>15</v>
+      </c>
+      <c r="N7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6084,6 +6105,9 @@
         <v>22</v>
       </c>
       <c r="M8" s="2">
+        <v>25</v>
+      </c>
+      <c r="N8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6125,6 +6149,9 @@
         <v>39</v>
       </c>
       <c r="M9" s="2">
+        <v>31</v>
+      </c>
+      <c r="N9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6166,6 +6193,9 @@
         <v>3</v>
       </c>
       <c r="M10" s="2">
+        <v>4</v>
+      </c>
+      <c r="N10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6207,6 +6237,9 @@
         <v>10</v>
       </c>
       <c r="M11" s="2">
+        <v>2</v>
+      </c>
+      <c r="N11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6248,6 +6281,9 @@
         <v>3</v>
       </c>
       <c r="M12" s="2">
+        <v>13</v>
+      </c>
+      <c r="N12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6289,6 +6325,9 @@
         <v>5</v>
       </c>
       <c r="M13" s="2">
+        <v>4</v>
+      </c>
+      <c r="N13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6330,6 +6369,9 @@
         <v>5</v>
       </c>
       <c r="M14" s="2">
+        <v>10</v>
+      </c>
+      <c r="N14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6371,6 +6413,9 @@
         <v>-19</v>
       </c>
       <c r="M15" s="2">
+        <v>15</v>
+      </c>
+      <c r="N15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6412,6 +6457,9 @@
         <v>6</v>
       </c>
       <c r="M16" s="2">
+        <v>4</v>
+      </c>
+      <c r="N16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6453,6 +6501,9 @@
         <v>8</v>
       </c>
       <c r="M17" s="2">
+        <v>3</v>
+      </c>
+      <c r="N17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6494,6 +6545,9 @@
         <v>4</v>
       </c>
       <c r="M18" s="2">
+        <v>9</v>
+      </c>
+      <c r="N18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6535,6 +6589,9 @@
         <v>8</v>
       </c>
       <c r="M19" s="2">
+        <v>10</v>
+      </c>
+      <c r="N19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6576,6 +6633,9 @@
         <v>8</v>
       </c>
       <c r="M20" s="2">
+        <v>6</v>
+      </c>
+      <c r="N20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6617,6 +6677,9 @@
         <v>8</v>
       </c>
       <c r="M21" s="2">
+        <v>3</v>
+      </c>
+      <c r="N21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6658,6 +6721,9 @@
         <v>1</v>
       </c>
       <c r="M22" s="2">
+        <v>-16</v>
+      </c>
+      <c r="N22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6699,6 +6765,9 @@
         <v>-17</v>
       </c>
       <c r="M23" s="2">
+        <v>-20</v>
+      </c>
+      <c r="N23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6756,6 +6825,9 @@
       <c r="L1" s="3">
         <v>11</v>
       </c>
+      <c r="M1" s="3">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6792,6 +6864,9 @@
         <v>71</v>
       </c>
       <c r="L2" s="2">
+        <v>38</v>
+      </c>
+      <c r="M2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6830,6 +6905,9 @@
         <v>71</v>
       </c>
       <c r="L3" s="2">
+        <v>71</v>
+      </c>
+      <c r="M3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6868,6 +6946,9 @@
         <v>79</v>
       </c>
       <c r="L4" s="2">
+        <v>59</v>
+      </c>
+      <c r="M4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6906,6 +6987,9 @@
         <v>42</v>
       </c>
       <c r="L5" s="2">
+        <v>71</v>
+      </c>
+      <c r="M5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6944,6 +7028,9 @@
         <v>19</v>
       </c>
       <c r="L6" s="2">
+        <v>10</v>
+      </c>
+      <c r="M6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6982,6 +7069,9 @@
         <v>15</v>
       </c>
       <c r="L7" s="2">
+        <v>10</v>
+      </c>
+      <c r="M7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7020,6 +7110,9 @@
         <v>15</v>
       </c>
       <c r="L8" s="2">
+        <v>47</v>
+      </c>
+      <c r="M8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7058,6 +7151,9 @@
         <v>19</v>
       </c>
       <c r="L9" s="2">
+        <v>29</v>
+      </c>
+      <c r="M9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7096,6 +7192,9 @@
         <v>-13</v>
       </c>
       <c r="L10" s="2">
+        <v>36</v>
+      </c>
+      <c r="M10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7134,6 +7233,9 @@
         <v>19</v>
       </c>
       <c r="L11" s="2">
+        <v>17</v>
+      </c>
+      <c r="M11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7172,6 +7274,9 @@
         <v>-17</v>
       </c>
       <c r="L12" s="2">
+        <v>-37</v>
+      </c>
+      <c r="M12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7227,6 +7332,9 @@
       <c r="M1" s="3">
         <v>11</v>
       </c>
+      <c r="N1" s="3">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -7268,6 +7376,9 @@
       <c r="M2" s="1">
         <v>25.8</v>
       </c>
+      <c r="N2" s="1">
+        <v>26.1</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -7309,6 +7420,9 @@
       <c r="M3" s="1">
         <v>24.7</v>
       </c>
+      <c r="N3" s="1">
+        <v>24.4</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -7350,6 +7464,9 @@
       <c r="M4" s="1">
         <v>28</v>
       </c>
+      <c r="N4" s="1">
+        <v>27.9</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -7391,6 +7508,9 @@
       <c r="M5" s="1">
         <v>25.6</v>
       </c>
+      <c r="N5" s="1">
+        <v>25.7</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -7432,6 +7552,9 @@
       <c r="M6" s="1">
         <v>27.7</v>
       </c>
+      <c r="N6" s="1">
+        <v>27.6</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -7473,6 +7596,9 @@
       <c r="M7" s="1">
         <v>13.9</v>
       </c>
+      <c r="N7" s="1">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -7514,6 +7640,9 @@
       <c r="M8" s="1">
         <v>24.9</v>
       </c>
+      <c r="N8" s="1">
+        <v>25</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -7555,6 +7684,9 @@
       <c r="M9" s="1">
         <v>23.6</v>
       </c>
+      <c r="N9" s="1">
+        <v>23.9</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -7596,6 +7728,9 @@
       <c r="M10" s="1">
         <v>6.4</v>
       </c>
+      <c r="N10" s="1">
+        <v>5.8</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -7637,6 +7772,9 @@
       <c r="M11" s="1">
         <v>10.2</v>
       </c>
+      <c r="N11" s="1">
+        <v>10</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -7678,6 +7816,9 @@
       <c r="M12" s="1">
         <v>9.7</v>
       </c>
+      <c r="N12" s="1">
+        <v>10.3</v>
+      </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -7719,6 +7860,9 @@
       <c r="M13" s="1">
         <v>7.4</v>
       </c>
+      <c r="N13" s="1">
+        <v>8</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -7760,6 +7904,9 @@
       <c r="M14" s="1">
         <v>5.6</v>
       </c>
+      <c r="N14" s="1">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -7801,6 +7948,9 @@
       <c r="M15" s="1">
         <v>3</v>
       </c>
+      <c r="N15" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -7842,6 +7992,9 @@
       <c r="M16" s="1">
         <v>10.5</v>
       </c>
+      <c r="N16" s="1">
+        <v>10.7</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -7883,6 +8036,9 @@
       <c r="M17" s="1">
         <v>7.4</v>
       </c>
+      <c r="N17" s="1">
+        <v>7.6</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -7924,6 +8080,9 @@
       <c r="M18" s="1">
         <v>3</v>
       </c>
+      <c r="N18" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -7965,6 +8124,9 @@
       <c r="M19" s="1">
         <v>7.2</v>
       </c>
+      <c r="N19" s="1">
+        <v>7.8</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -8006,6 +8168,9 @@
       <c r="M20" s="1">
         <v>12.8</v>
       </c>
+      <c r="N20" s="1">
+        <v>13</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -8047,6 +8212,9 @@
       <c r="M21" s="1">
         <v>11</v>
       </c>
+      <c r="N21" s="1">
+        <v>11.2</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -8088,6 +8256,9 @@
       <c r="M22" s="1">
         <v>3</v>
       </c>
+      <c r="N22" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -8128,6 +8299,9 @@
       </c>
       <c r="M23" s="1">
         <v>4.4</v>
+      </c>
+      <c r="N23" s="1">
+        <v>3.8</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -8184,6 +8358,9 @@
       <c r="L1" s="3">
         <v>11</v>
       </c>
+      <c r="M1" s="3">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -8222,6 +8399,9 @@
       <c r="L2" s="1">
         <v>30.7</v>
       </c>
+      <c r="M2" s="1">
+        <v>31</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -8260,6 +8440,9 @@
       <c r="L3" s="1">
         <v>26.3</v>
       </c>
+      <c r="M3" s="1">
+        <v>26.6</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -8298,6 +8481,9 @@
       <c r="L4" s="1">
         <v>30.6</v>
       </c>
+      <c r="M4" s="1">
+        <v>30.9</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -8336,6 +8522,9 @@
       <c r="L5" s="1">
         <v>32.3</v>
       </c>
+      <c r="M5" s="1">
+        <v>32.6</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -8374,6 +8563,9 @@
       <c r="L6" s="1">
         <v>13.2</v>
       </c>
+      <c r="M6" s="1">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -8412,6 +8604,9 @@
       <c r="L7" s="1">
         <v>12.3</v>
       </c>
+      <c r="M7" s="1">
+        <v>12.9</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -8450,6 +8645,9 @@
       <c r="L8" s="1">
         <v>11.4</v>
       </c>
+      <c r="M8" s="1">
+        <v>12</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -8488,6 +8686,9 @@
       <c r="L9" s="1">
         <v>5.1</v>
       </c>
+      <c r="M9" s="1">
+        <v>5.7</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -8526,6 +8727,9 @@
       <c r="L10" s="1">
         <v>18.5</v>
       </c>
+      <c r="M10" s="1">
+        <v>18.8</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -8564,6 +8768,9 @@
       <c r="L11" s="1">
         <v>6.2</v>
       </c>
+      <c r="M11" s="1">
+        <v>6.8</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -8601,6 +8808,9 @@
       </c>
       <c r="L12" s="1">
         <v>3.6</v>
+      </c>
+      <c r="M12" s="1">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refreshed team after HAD not racing
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -6063,9 +6063,7 @@
       <c r="M7" s="2">
         <v>15</v>
       </c>
-      <c r="N7" s="2">
-        <v>0</v>
-      </c>
+      <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
@@ -6283,9 +6281,7 @@
       <c r="M12" s="2">
         <v>13</v>
       </c>
-      <c r="N12" s="2">
-        <v>0</v>
-      </c>
+      <c r="N12" s="2"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="2" t="s">
@@ -6772,9 +6768,27 @@
       </c>
     </row>
     <row r="24" spans="1:3">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="C24" s="2"/>
+      <c r="N24" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N25" s="2">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7596,9 +7610,7 @@
       <c r="M7" s="1">
         <v>13.9</v>
       </c>
-      <c r="N7" s="1">
-        <v>14.5</v>
-      </c>
+      <c r="N7" s="1"/>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="2" t="s">
@@ -7816,9 +7828,7 @@
       <c r="M12" s="1">
         <v>9.7</v>
       </c>
-      <c r="N12" s="1">
-        <v>10.3</v>
-      </c>
+      <c r="N12" s="1"/>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="2" t="s">
@@ -8305,9 +8315,27 @@
       </c>
     </row>
     <row r="24" spans="1:5">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
+      <c r="A24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="C24" s="2"/>
+      <c r="N24" s="1">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="N25" s="1">
+        <v>10.3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated points and prices for race 12
</commit_message>
<xml_diff>
--- a/data/f1_fantasy_archive.xlsx
+++ b/data/f1_fantasy_archive.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E98229F0-2B07-4F07-A68F-AC4F3D4F854E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView activeTab="12" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
+    <workbookView activeTab="14" firstSheet="10" windowHeight="15840" windowWidth="29040" xWindow="-120" xr2:uid="{5075C4C2-DC0E-48A5-BDF1-482703F248E6}" yWindow="-120"/>
   </bookViews>
   <sheets>
     <sheet name="2023 Drivers Points" sheetId="1" r:id="rId1"/>
@@ -5802,6 +5802,9 @@
       <c r="N1" s="3">
         <v>12</v>
       </c>
+      <c r="O1" s="3">
+        <v>13</v>
+      </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="2" t="s">
@@ -5844,6 +5847,9 @@
         <v>37</v>
       </c>
       <c r="N2" s="2">
+        <v>57</v>
+      </c>
+      <c r="O2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5888,6 +5894,9 @@
         <v>-11</v>
       </c>
       <c r="N3" s="2">
+        <v>21</v>
+      </c>
+      <c r="O3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5932,6 +5941,9 @@
         <v>23</v>
       </c>
       <c r="N4" s="2">
+        <v>32</v>
+      </c>
+      <c r="O4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -5976,6 +5988,9 @@
         <v>28</v>
       </c>
       <c r="N5" s="2">
+        <v>37</v>
+      </c>
+      <c r="O5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6020,6 +6035,9 @@
         <v>39</v>
       </c>
       <c r="N6" s="2">
+        <v>-13</v>
+      </c>
+      <c r="O6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6064,6 +6082,7 @@
         <v>15</v>
       </c>
       <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="2" t="s">
@@ -6106,6 +6125,9 @@
         <v>25</v>
       </c>
       <c r="N8" s="2">
+        <v>23</v>
+      </c>
+      <c r="O8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6150,6 +6172,9 @@
         <v>31</v>
       </c>
       <c r="N9" s="2">
+        <v>39</v>
+      </c>
+      <c r="O9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6194,6 +6219,9 @@
         <v>4</v>
       </c>
       <c r="N10" s="2">
+        <v>2</v>
+      </c>
+      <c r="O10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6238,6 +6266,9 @@
         <v>2</v>
       </c>
       <c r="N11" s="2">
+        <v>7</v>
+      </c>
+      <c r="O11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6282,6 +6313,7 @@
         <v>13</v>
       </c>
       <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="2" t="s">
@@ -6324,6 +6356,9 @@
         <v>4</v>
       </c>
       <c r="N13" s="2">
+        <v>7</v>
+      </c>
+      <c r="O13" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6368,6 +6403,9 @@
         <v>10</v>
       </c>
       <c r="N14" s="2">
+        <v>24</v>
+      </c>
+      <c r="O14" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6412,6 +6450,9 @@
         <v>15</v>
       </c>
       <c r="N15" s="2">
+        <v>-10</v>
+      </c>
+      <c r="O15" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6456,6 +6497,9 @@
         <v>4</v>
       </c>
       <c r="N16" s="2">
+        <v>-10</v>
+      </c>
+      <c r="O16" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6500,6 +6544,9 @@
         <v>3</v>
       </c>
       <c r="N17" s="2">
+        <v>-13</v>
+      </c>
+      <c r="O17" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6544,6 +6591,9 @@
         <v>9</v>
       </c>
       <c r="N18" s="2">
+        <v>5</v>
+      </c>
+      <c r="O18" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6588,6 +6638,9 @@
         <v>10</v>
       </c>
       <c r="N19" s="2">
+        <v>5</v>
+      </c>
+      <c r="O19" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6632,6 +6685,9 @@
         <v>6</v>
       </c>
       <c r="N20" s="2">
+        <v>8</v>
+      </c>
+      <c r="O20" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6676,6 +6732,9 @@
         <v>3</v>
       </c>
       <c r="N21" s="2">
+        <v>6</v>
+      </c>
+      <c r="O21" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6720,6 +6779,9 @@
         <v>-16</v>
       </c>
       <c r="N22" s="2">
+        <v>-18</v>
+      </c>
+      <c r="O22" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6764,6 +6826,9 @@
         <v>-20</v>
       </c>
       <c r="N23" s="2">
+        <v>8</v>
+      </c>
+      <c r="O23" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6776,6 +6841,9 @@
       </c>
       <c r="C24" s="2"/>
       <c r="N24" s="2">
+        <v>12</v>
+      </c>
+      <c r="O24" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6787,6 +6855,9 @@
         <v>35</v>
       </c>
       <c r="N25" s="2">
+        <v>5</v>
+      </c>
+      <c r="O25" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6842,6 +6913,9 @@
       <c r="M1" s="3">
         <v>12</v>
       </c>
+      <c r="N1" s="3">
+        <v>13</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -6881,6 +6955,9 @@
         <v>38</v>
       </c>
       <c r="M2" s="2">
+        <v>80</v>
+      </c>
+      <c r="N2" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6922,6 +6999,9 @@
         <v>71</v>
       </c>
       <c r="M3" s="2">
+        <v>74</v>
+      </c>
+      <c r="N3" s="2">
         <v>0</v>
       </c>
     </row>
@@ -6963,6 +7043,9 @@
         <v>59</v>
       </c>
       <c r="M4" s="2">
+        <v>11</v>
+      </c>
+      <c r="N4" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7004,6 +7087,9 @@
         <v>71</v>
       </c>
       <c r="M5" s="2">
+        <v>84</v>
+      </c>
+      <c r="N5" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7045,6 +7131,9 @@
         <v>10</v>
       </c>
       <c r="M6" s="2">
+        <v>15</v>
+      </c>
+      <c r="N6" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7086,6 +7175,9 @@
         <v>10</v>
       </c>
       <c r="M7" s="2">
+        <v>-20</v>
+      </c>
+      <c r="N7" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7127,6 +7219,9 @@
         <v>47</v>
       </c>
       <c r="M8" s="2">
+        <v>22</v>
+      </c>
+      <c r="N8" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7168,6 +7263,9 @@
         <v>29</v>
       </c>
       <c r="M9" s="2">
+        <v>25</v>
+      </c>
+      <c r="N9" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7209,6 +7307,9 @@
         <v>36</v>
       </c>
       <c r="M10" s="2">
+        <v>18</v>
+      </c>
+      <c r="N10" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7250,6 +7351,9 @@
         <v>17</v>
       </c>
       <c r="M11" s="2">
+        <v>19</v>
+      </c>
+      <c r="N11" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7291,6 +7395,9 @@
         <v>-37</v>
       </c>
       <c r="M12" s="2">
+        <v>-9</v>
+      </c>
+      <c r="N12" s="2">
         <v>0</v>
       </c>
     </row>
@@ -7349,6 +7456,9 @@
       <c r="N1" s="3">
         <v>12</v>
       </c>
+      <c r="O1" s="3">
+        <v>13</v>
+      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="2" t="s">
@@ -7393,6 +7503,9 @@
       <c r="N2" s="1">
         <v>26.1</v>
       </c>
+      <c r="O2" s="1">
+        <v>26.4</v>
+      </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
@@ -7437,6 +7550,9 @@
       <c r="N3" s="1">
         <v>24.4</v>
       </c>
+      <c r="O3" s="1">
+        <v>24.1</v>
+      </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="2" t="s">
@@ -7481,6 +7597,9 @@
       <c r="N4" s="1">
         <v>27.9</v>
       </c>
+      <c r="O4" s="1">
+        <v>27.6</v>
+      </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="2" t="s">
@@ -7525,6 +7644,9 @@
       <c r="N5" s="1">
         <v>25.7</v>
       </c>
+      <c r="O5" s="1">
+        <v>26</v>
+      </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="2" t="s">
@@ -7569,6 +7691,9 @@
       <c r="N6" s="1">
         <v>27.6</v>
       </c>
+      <c r="O6" s="1">
+        <v>27.5</v>
+      </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="2" t="s">
@@ -7655,6 +7780,9 @@
       <c r="N8" s="1">
         <v>25</v>
       </c>
+      <c r="O8" s="1">
+        <v>25.1</v>
+      </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="2" t="s">
@@ -7699,6 +7827,9 @@
       <c r="N9" s="1">
         <v>23.9</v>
       </c>
+      <c r="O9" s="1">
+        <v>24.2</v>
+      </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="2" t="s">
@@ -7743,6 +7874,9 @@
       <c r="N10" s="1">
         <v>5.8</v>
       </c>
+      <c r="O10" s="1">
+        <v>5.2</v>
+      </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="2" t="s">
@@ -7787,6 +7921,9 @@
       <c r="N11" s="1">
         <v>10</v>
       </c>
+      <c r="O11" s="1">
+        <v>9.8</v>
+      </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="2" t="s">
@@ -7873,6 +8010,9 @@
       <c r="N13" s="1">
         <v>8</v>
       </c>
+      <c r="O13" s="1">
+        <v>7.8</v>
+      </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="2" t="s">
@@ -7917,6 +8057,9 @@
       <c r="N14" s="1">
         <v>6.2</v>
       </c>
+      <c r="O14" s="1">
+        <v>6.8</v>
+      </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="2" t="s">
@@ -7961,6 +8104,9 @@
       <c r="N15" s="1">
         <v>3</v>
       </c>
+      <c r="O15" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="2" t="s">
@@ -8005,6 +8151,9 @@
       <c r="N16" s="1">
         <v>10.7</v>
       </c>
+      <c r="O16" s="1">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="2" t="s">
@@ -8049,6 +8198,9 @@
       <c r="N17" s="1">
         <v>7.6</v>
       </c>
+      <c r="O17" s="1">
+        <v>7</v>
+      </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
@@ -8093,6 +8245,9 @@
       <c r="N18" s="1">
         <v>3</v>
       </c>
+      <c r="O18" s="1">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
@@ -8137,6 +8292,9 @@
       <c r="N19" s="1">
         <v>7.8</v>
       </c>
+      <c r="O19" s="1">
+        <v>8</v>
+      </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
@@ -8181,6 +8339,9 @@
       <c r="N20" s="1">
         <v>13</v>
       </c>
+      <c r="O20" s="1">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="2" t="s">
@@ -8225,6 +8386,9 @@
       <c r="N21" s="1">
         <v>11.2</v>
       </c>
+      <c r="O21" s="1">
+        <v>10.6</v>
+      </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
@@ -8269,6 +8433,9 @@
       <c r="N22" s="1">
         <v>3</v>
       </c>
+      <c r="O22" s="1">
+        <v>3</v>
+      </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="2" t="s">
@@ -8313,6 +8480,9 @@
       <c r="N23" s="1">
         <v>3.8</v>
       </c>
+      <c r="O23" s="1">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="2" t="s">
@@ -8325,6 +8495,9 @@
       <c r="N24" s="1">
         <v>14.5</v>
       </c>
+      <c r="O24" s="1">
+        <v>14.3</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="s">
@@ -8335,6 +8508,9 @@
       </c>
       <c r="N25" s="1">
         <v>10.3</v>
+      </c>
+      <c r="O25" s="1">
+        <v>9.7</v>
       </c>
     </row>
   </sheetData>
@@ -8389,6 +8565,9 @@
       <c r="M1" s="3">
         <v>12</v>
       </c>
+      <c r="N1" s="3">
+        <v>13</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="2" t="s">
@@ -8430,6 +8609,9 @@
       <c r="M2" s="1">
         <v>31</v>
       </c>
+      <c r="N2" s="1">
+        <v>31.3</v>
+      </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="2" t="s">
@@ -8471,6 +8653,9 @@
       <c r="M3" s="1">
         <v>26.6</v>
       </c>
+      <c r="N3" s="1">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="2" t="s">
@@ -8512,6 +8697,9 @@
       <c r="M4" s="1">
         <v>30.9</v>
       </c>
+      <c r="N4" s="1">
+        <v>31.2</v>
+      </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="2" t="s">
@@ -8553,6 +8741,9 @@
       <c r="M5" s="1">
         <v>32.6</v>
       </c>
+      <c r="N5" s="1">
+        <v>32.9</v>
+      </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="2" t="s">
@@ -8594,6 +8785,9 @@
       <c r="M6" s="1">
         <v>13</v>
       </c>
+      <c r="N6" s="1">
+        <v>13.2</v>
+      </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="2" t="s">
@@ -8635,6 +8829,9 @@
       <c r="M7" s="1">
         <v>12.9</v>
       </c>
+      <c r="N7" s="1">
+        <v>13.5</v>
+      </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="2" t="s">
@@ -8676,6 +8873,9 @@
       <c r="M8" s="1">
         <v>12</v>
       </c>
+      <c r="N8" s="1">
+        <v>11.4</v>
+      </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="2" t="s">
@@ -8717,6 +8917,9 @@
       <c r="M9" s="1">
         <v>5.7</v>
       </c>
+      <c r="N9" s="1">
+        <v>6.3</v>
+      </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="2" t="s">
@@ -8758,6 +8961,9 @@
       <c r="M10" s="1">
         <v>18.8</v>
       </c>
+      <c r="N10" s="1">
+        <v>18.9</v>
+      </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
@@ -8799,6 +9005,9 @@
       <c r="M11" s="1">
         <v>6.8</v>
       </c>
+      <c r="N11" s="1">
+        <v>7.4</v>
+      </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" s="2" t="s">
@@ -8838,6 +9047,9 @@
         <v>3.6</v>
       </c>
       <c r="M12" s="1">
+        <v>3</v>
+      </c>
+      <c r="N12" s="1">
         <v>3</v>
       </c>
     </row>

</xml_diff>